<commit_message>
D5 for Table 3 modified to have combinations of ATC IV level instead of single ATC IV level and results based on simulated data updated
</commit_message>
<xml_diff>
--- a/i_test/test_D6_Tabella_3_2025/g_output/D6_Table_3.xlsx
+++ b/i_test/test_D6_Tabella_3_2025/g_output/D6_Table_3.xlsx
@@ -416,22 +416,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>3035</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>960</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>1055</t>
         </is>
       </c>
     </row>
@@ -443,22 +443,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>25 (55,6%)</t>
+          <t>1.507 (49,7%)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6 (66,7%)</t>
+          <t>497 (48,7%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8 (42,1%)</t>
+          <t>493 (51,4%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11 (64,7%)</t>
+          <t>517 (49,0%)</t>
         </is>
       </c>
     </row>
@@ -470,22 +470,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>13 (28,9%)</t>
+          <t>1.051 (34,6%)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3 (33,3%)</t>
+          <t>357 (35,0%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5 (26,3%)</t>
+          <t>342 (35,6%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>5 (29,4%)</t>
+          <t>352 (33,4%)</t>
         </is>
       </c>
     </row>
@@ -497,22 +497,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19 (42,2%)</t>
+          <t>998 (32,9%)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5 (55,6%)</t>
+          <t>330 (32,4%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (31,6%)</t>
+          <t>306 (31,9%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>8 (47,1%)</t>
+          <t>362 (34,3%)</t>
         </is>
       </c>
     </row>
@@ -524,22 +524,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>13 (28,9%)</t>
+          <t>986 (32,5%)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1 (11,1%)</t>
+          <t>333 (32,6%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>8 (42,1%)</t>
+          <t>312 (32,5%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4 (23,5%)</t>
+          <t>341 (32,3%)</t>
         </is>
       </c>
     </row>
@@ -551,22 +551,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4 (8,9%)</t>
+          <t>2.030 (66,9%)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3 (33,3%)</t>
+          <t>692 (67,8%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (5,3%)</t>
+          <t>638 (66,5%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0 (0,0%)</t>
+          <t>700 (66,4%)</t>
         </is>
       </c>
     </row>
@@ -585,22 +585,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>28 (62,2%)</t>
+          <t>1.485 (48,9%)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>7 (77,8%)</t>
+          <t>500 (49,0%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11 (57,9%)</t>
+          <t>454 (47,3%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>10 (58,8%)</t>
+          <t>531 (50,3%)</t>
         </is>
       </c>
     </row>
@@ -612,22 +612,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>5 (11,1%)</t>
+          <t>541 (17,8%)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1 (11,1%)</t>
+          <t>171 (16,8%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1 (5,3%)</t>
+          <t>161 (16,8%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>3 (17,6%)</t>
+          <t>209 (19,8%)</t>
         </is>
       </c>
     </row>
@@ -639,22 +639,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>27 (60,0%)</t>
+          <t>1.978 (65,2%)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>9 (100,0%)</t>
+          <t>665 (65,2%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10 (52,6%)</t>
+          <t>640 (66,7%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>8 (47,1%)</t>
+          <t>673 (63,8%)</t>
         </is>
       </c>
     </row>
@@ -666,22 +666,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14 (31,1%)</t>
+          <t>1.710 (56,3%)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3 (33,3%)</t>
+          <t>571 (56,0%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5 (26,3%)</t>
+          <t>549 (57,2%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>6 (35,3%)</t>
+          <t>590 (55,9%)</t>
         </is>
       </c>
     </row>
@@ -700,22 +700,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>A10BD15 20 (44,4%)</t>
+          <t>J10JE54 201 (6,6%)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>A10BD15 7 (77,8%)</t>
+          <t>A10BD07 77 (7,5%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>A10AE56 11 (57,9%)</t>
+          <t>B10BX16 74 (7,7%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>A10BJ 9 (52,9%)</t>
+          <t>J10JE54 84 (8,0%)</t>
         </is>
       </c>
     </row>
@@ -727,22 +727,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>A10BD07 20 (44,4%)</t>
+          <t>B10BD19 199 (6,6%)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>A10BD24 5 (55,6%)</t>
+          <t>C10BD20 75 (7,4%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>A10BD09 10 (52,6%)</t>
+          <t>D10DE54 68 (7,1%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>A10BD15 9 (52,9%)</t>
+          <t>D10BD07 79 (7,5%)</t>
         </is>
       </c>
     </row>
@@ -754,22 +754,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>A10AE56 20 (44,4%)</t>
+          <t>A10BD07 194 (6,4%)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A10BD16 4 (44,4%)</t>
+          <t>A10BD09 73 (7,2%)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>A10BD07 9 (47,4%)</t>
+          <t>C10BD23 67 (7,0%)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>A10BH 9 (52,9%)</t>
+          <t>A10BH02 78 (7,4%)</t>
         </is>
       </c>
     </row>
@@ -781,22 +781,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>A10BH 19 (42,2%)</t>
+          <t>B10AE54 193 (6,4%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>A10BH 4 (44,4%)</t>
+          <t>J10BD20 72 (7,1%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>A10AE54 8 (42,1%)</t>
+          <t>B10BD19 67 (7,0%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>A10BD21 8 (47,1%)</t>
+          <t>B10BD20 77 (7,3%)</t>
         </is>
       </c>
     </row>
@@ -808,22 +808,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>A10BD16 18 (40,0%)</t>
+          <t>B10BX16 193 (6,4%)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>A10BD21 4 (44,4%)</t>
+          <t>A10BD21 72 (7,1%)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>A10BD11 8 (42,1%)</t>
+          <t>C10BD11 66 (6,9%)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>A10BD08 8 (47,1%)</t>
+          <t>B10BD15 73 (6,9%)</t>
         </is>
       </c>
     </row>
@@ -842,22 +842,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>A10BD 45 (100,0%)</t>
+          <t>A10BD B10BD C10BD J10BD M10BD 15 (0,5%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>A10BD 9 (100,0%)</t>
+          <t>A10BD B10BD C10BD J10BD M10BD 4 (0,4%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>A10BD 19 (100,0%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD 6 (0,6%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>A10BD 17 (100,0%)</t>
+          <t>A10BD B10BD C10BD J10BD M10BD 7 (0,7%)</t>
         </is>
       </c>
     </row>
@@ -869,22 +869,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>A10AE 27 (60,0%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD 12 (0,4%)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>A10BH 4 (44,4%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD 4 (0,4%)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>A10AE 13 (68,4%)</t>
+          <t>A10BD C10BD D10BD J10BD M10BD 4 (0,4%)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>A10AE 11 (64,7%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD M10BD 5 (0,5%)</t>
         </is>
       </c>
     </row>
@@ -896,22 +896,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>A10BH 16 (35,6%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD M10BD 10 (0,3%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>A10AE 3 (33,3%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD M10BD M10ME 2 (0,2%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>A10BH 5 (26,3%)</t>
+          <t>A10BD B10BD C10BD J10BD M10BD 4 (0,4%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>A10BJ 7 (41,2%)</t>
+          <t>B10BD C10BD D10BD J10BD M10BD 3 (0,3%)</t>
         </is>
       </c>
     </row>
@@ -923,22 +923,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>A10BJ 15 (33,3%)</t>
+          <t>B10BD C10BD D10BD J10BD M10BD 7 (0,2%)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>A10BJ 3 (33,3%)</t>
+          <t>A10BD B10BD C10BD C10BK J10BD M10BD 2 (0,2%)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>A10BK 5 (26,3%)</t>
+          <t>B10BD C10BD D10BD J10BD M10BD 4 (0,4%)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>A10BH 7 (41,2%)</t>
+          <t>A10BD B10BD C10BD D10BD M10BD 3 (0,3%)</t>
         </is>
       </c>
     </row>
@@ -950,22 +950,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>A10BK 12 (26,7%)</t>
+          <t>A10BD C10BD D10BD J10BD M10BD 7 (0,2%)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>A10BX 2 (22,2%)</t>
+          <t>A10BD B10BD C10BD D10BD D10DE M10BD 2 (0,2%)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>A10BJ 5 (26,3%)</t>
+          <t>A10AE B10BD C10BD D10BD J10BD M10BD 3 (0,3%)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>A10BK 6 (35,3%)</t>
+          <t>B10BJ C10BD D10BD J10BD M10BD 2 (0,2%)</t>
         </is>
       </c>
     </row>

</xml_diff>